<commit_message>
News Scraper: Final Fixed V.1.0
</commit_message>
<xml_diff>
--- a/data/processed/news.xlsx
+++ b/data/processed/news.xlsx
@@ -1526,7 +1526,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Lancashire bring in Pakistan spinner Noman</t>
+          <t>Send your cricket data questions to BBC Sport &amp; CricViz</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1536,159 +1536,159 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Lancashire sign Pakistan spinner Noman Ali for the final six games of the County Championship season.</t>
+          <t>Send your cricket data questions to BBC Sport and we will get CricViz to answer a selection of them.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c9d893pzv34o</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/cz6459x3zw0o</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-08-06 10:36:06</t>
+          <t>2026-08-19 16:03:53</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Test Match Special Podcast</t>
+          <t>Lancashire bring in Pakistan spinner Noman</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Unknown Author</t>
+          <t>BBC Sport</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Cricket analysis with Sir Alastair Cook, Steven Finn and Alex Hartley.</t>
+          <t>Lancashire sign Pakistan spinner Noman Ali for the final six games of the County Championship season.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sounds/play/p0p2h3c2?at_campaign=rss</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c9d893pzv34o</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-08-03 21:17:00</t>
+          <t>2026-08-06 10:36:06</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Greaves takes 5-0 in incredible Test bowling spell</t>
+          <t>Test Match Special Podcast</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Timothy Abraham</t>
+          <t>Unknown Author</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>West Indies all-rounder Justin Greaves takes five wickets without conceding a run during an incredible spell of bowling on day three of the first Test against Pakistan.</t>
+          <t>Cricket analysis with Sir Alastair Cook, Steven Finn and Alex Hartley.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/cx2rjv5599go</t>
+          <t>https://www.bbc.co.uk/sounds/play/p0p2h3c2?at_campaign=rss</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-07-27 22:27:14</t>
+          <t>2026-08-03 21:17:00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>England hopeful Gay will be fit for Pakistan Test</t>
+          <t>Greaves takes 5-0 in incredible Test bowling spell</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Stephan Shemilt</t>
+          <t>Timothy Abraham</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Opener Emilio Gay will have further treatment on a shoulder injury this week with England hopeful he will be fit for the first Test against Pakistan.</t>
+          <t>West Indies all-rounder Justin Greaves takes five wickets without conceding a run during an incredible spell of bowling on day three of the first Test against Pakistan.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/cpd75xqj99go</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/cx2rjv5599go</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-08-10 15:36:34</t>
+          <t>2026-07-27 22:27:14</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>'Pressure will follow him' - Rocky Flintoff faces up to tests ahead</t>
+          <t>England hopeful Gay will be fit for Pakistan Test</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Matthew Henry</t>
+          <t>Stephan Shemilt</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>With one former England coach calling for Rocky Flintoff to be "fast-tracked" to international cricket, what should be next for the talented teenager?</t>
+          <t>Opener Emilio Gay will have further treatment on a shoulder injury this week with England hopeful he will be fit for the first Test against Pakistan.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c9342w19n81o</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/cpd75xqj99go</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-08-15 08:23:21</t>
+          <t>2026-08-10 15:36:34</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Brook's time will come as Test captain - McCullum</t>
+          <t>'Pressure will follow him' - Rocky Flintoff faces up to tests ahead</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ffion Wynne</t>
+          <t>Matthew Henry</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>England white-ball coach Brendon McCullum backs Harry Brook as a future captain but says Joe Root will do an "amazing job" in his second stint.</t>
+          <t>With one former England coach calling for Rocky Flintoff to be "fast-tracked" to international cricket, what should be next for the talented teenager?</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c39epglkg8mo</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c9342w19n81o</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-08-06 19:02:55</t>
+          <t>2026-08-15 08:23:21</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Bethell ruled out of The Hundred with knee injury</t>
+          <t>Brook's time will come as Test captain - McCullum</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1698,322 +1698,322 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>England all-rounder Jacob Bethell, who was due to captain Birmingham Phoenix, is ruled out of The Hundred with a knee injury.</t>
+          <t>England white-ball coach Brendon McCullum backs Harry Brook as a future captain but says Joe Root will do an "amazing job" in his second stint.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c8jn9p49n99o</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c39epglkg8mo</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-07-21 12:50:40</t>
+          <t>2026-08-06 19:02:55</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Seamer Randell joins Derbyshire for rest of season</t>
+          <t>Bethell ruled out of The Hundred with knee injury</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Andrew Aloia</t>
+          <t>Ffion Wynne</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Derbyshire sign history-making seam bowler Brett Randell for the remainder of the County Championship season.</t>
+          <t>England all-rounder Jacob Bethell, who was due to captain Birmingham Phoenix, is ruled out of The Hundred with a knee injury.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c20e27rrw9go</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c8jn9p49n99o</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-08-13 11:54:07</t>
+          <t>2026-07-21 12:50:40</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Lomror joins Surrey for County Championship finale</t>
+          <t>Seamer Randell joins Derbyshire for rest of season</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>BBC Sport</t>
+          <t>Andrew Aloia</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Surrey sign Indian batter Mahipal Lomror for the final six County Championship games of the 2026 season.</t>
+          <t>Derbyshire sign history-making seam bowler Brett Randell for the remainder of the County Championship season.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c74gkgy5q19o</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c20e27rrw9go</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-08-18 14:25:53</t>
+          <t>2026-08-13 11:54:07</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Warner fined for drink-driving &amp; must fit interlock device to car</t>
+          <t>Lomror joins Surrey for County Championship finale</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Adwaidh Rajan</t>
+          <t>BBC Sport</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Former Australia batter David Warner is convicted and fined for drink-driving following a random breath test in April.</t>
+          <t>Surrey sign Indian batter Mahipal Lomror for the final six County Championship games of the 2026 season.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c8dn353gjryo</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c74gkgy5q19o</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-08-18 07:55:59</t>
+          <t>2026-08-18 14:25:53</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Trescothick chat helps Buttler find form for T20 record</t>
+          <t>Warner fined for drink-driving &amp; must fit interlock device to car</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Mike Peter</t>
+          <t>Adwaidh Rajan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Jos Buttler says a conversation with England batting coach Marcus Trescothick helped him rediscover the form that took his past the all-time T20 run-scoring record.</t>
+          <t>Former Australia batter David Warner is convicted and fined for drink-driving following a random breath test in April.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/c3v0ed04w2qo</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c8dn353gjryo</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-08-07 13:49:44</t>
+          <t>2026-08-18 07:55:59</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ambitious Yorkshire strengthen with Arlott signing</t>
+          <t>Trescothick chat helps Buttler find form for T20 record</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>BBC Sport</t>
+          <t>Mike Peter</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Yorkshire sign England bowler Em Arlott from Warwickshire on a three-year-contract, starting next season.</t>
+          <t>Jos Buttler says a conversation with England batting coach Marcus Trescothick helped him rediscover the form that took his past the all-time T20 run-scoring record.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/cj4knvwxg9eo</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/c3v0ed04w2qo</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-07-24 09:46:19</t>
+          <t>2026-08-07 13:49:44</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Only wins can stop England's curfew hokey-cokey</t>
+          <t>Ambitious Yorkshire strengthen with Arlott signing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Stephan Shemilt</t>
+          <t>BBC Sport</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>England have scrapped their midnight curfew seven months after introducing it. Now, only wins will repair the reputational damage they have sustained, says Stephan Shemilt.</t>
+          <t>Yorkshire sign England bowler Em Arlott from Warwickshire on a three-year-contract, starting next season.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.bbc.co.uk/sport/cricket/articles/czjl2pelp1go</t>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/cj4knvwxg9eo</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-08-13 05:22:07</t>
+          <t>2026-07-24 09:46:19</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>Only wins can stop England's curfew hokey-cokey</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Stephan Shemilt</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>England have scrapped their midnight curfew seven months after introducing it. Now, only wins will repair the reputational damage they have sustained, says Stephan Shemilt.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.bbc.co.uk/sport/cricket/articles/czjl2pelp1go</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-08-13 05:22:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>Taliban authorities mark five years ruling Afghanistan</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>Henry Oduah</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Hundreds of Afghans gathered around a square beside the former US embassy, with men, boys and young girls packed into pickup trucks and waving white Taliban government flags.
 The post Taliban authorities mark five years ruling Afghanistan appeared first on Va…</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>https://www.vanguardngr.com/2026/08/taliban-authorities-mark-five-years-ruling-afghanistan/</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>2026-08-15 08:18:15</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>'You let BJP, Congress speak, but not us': Akhilesh Yadav erupts in Lok Sabha over NEET discussion</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>TIMESOFINDIA.COM</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Samajwadi Party chief Akhilesh Yadav accused the Lok Sabha Speaker of unfair treatment. He stated his party was denied a chance to speak on the NEET paper leak. The government and Congress were allowed to present their views while his party was not. Yadav ins…</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>https://timesofindia.indiatimes.com/india/you-let-bjp-congress-speak-but-not-us-akhilesh-yadav-erupts-in-lok-sabha-over-neet-discussion/articleshow/132554920.cms</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2026-07-22 08:51:33</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Fractured finger rules out Masood for the 2nd cricket test against West Indies</t>
+          <t>'You let BJP, Congress speak, but not us': Akhilesh Yadav erupts in Lok Sabha over NEET discussion</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Associated Press</t>
+          <t>TIMESOFINDIA.COM</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Pakistan in-form batter Shan Masood was ruled out of the second cricket test against the West Indies due to a fractured left index finger. Masood was the only bright batting spot in Pakistan’s 90-run defeat in the first test at Trinidad when the left-hander s…</t>
+          <t>Samajwadi Party chief Akhilesh Yadav accused the Lok Sabha Speaker of unfair treatment. He stated his party was denied a chance to speak on the NEET paper leak. The government and Congress were allowed to present their views while his party was not. Yadav ins…</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/fractured-finger-rules-masood-2nd-051738603.html</t>
+          <t>https://timesofindia.indiatimes.com/india/you-let-bjp-congress-speak-but-not-us-akhilesh-yadav-erupts-in-lok-sabha-over-neet-discussion/articleshow/132554920.cms</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-07-31 05:17:38</t>
+          <t>2026-07-22 08:51:33</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>'Darkly comical': Cricket world baffled as Pakistan drop 'best bowler' Mohammad Abbas for WI 2nd Test over 'conditions'</t>
+          <t>Fractured finger rules out Masood for the 2nd cricket test against West Indies</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Deepanjan Mitra</t>
+          <t>Associated Press</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>With the second Test between Pakistan and the Windies going in full fury, the whole cricket world remains confused about the sudden dropping of Mohammed Abba...</t>
+          <t>Pakistan in-form batter Shan Masood was ruled out of the second cricket test against the West Indies due to a fractured left index finger. Masood was the only bright batting spot in Pakistan’s 90-run defeat in the first test at Trinidad when the left-hander s…</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/cricket-world-pakistan-drop-best-bowler-mohammad-abbas-wi-test-conditions/802d5cc242191ee7d8a95402</t>
+          <t>https://sports.yahoo.com/articles/fractured-finger-rules-masood-2nd-051738603.html</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-08-02 18:40:43</t>
+          <t>2026-07-31 05:17:38</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Shoaib Akhtar likens himself to Brazilian icon Ronaldo Nazario if he swapped Pakistan cricket to play football</t>
+          <t>'Darkly comical': Cricket world baffled as Pakistan drop 'best bowler' Mohammad Abbas for WI 2nd Test over 'conditions'</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Soham Mukherjee</t>
+          <t>Deepanjan Mitra</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Former Pakistan speedster Shoaib Akhtar claims he would have played like Brazilian legend Ronaldo Nazario had he chosen football over international cricket.</t>
+          <t>With the second Test between Pakistan and the Windies going in full fury, the whole cricket world remains confused about the sudden dropping of Mohammed Abba...</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/shoaib-akhtar-brazilian-ronaldo-nazario-pakistan-cricket-football/a8907afaa907e84e21f7aea7</t>
+          <t>https://www.cricketnews.com/en/cricket/news/cricket-world-pakistan-drop-best-bowler-mohammad-abbas-wi-test-conditions/802d5cc242191ee7d8a95402</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-07-25 03:52:34</t>
+          <t>2026-08-02 18:40:43</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Tarouba, Trinidad weather forecast: Day-by-Day rain chances for West Indies vs Pakistan 1st Test 2026</t>
+          <t>Shoaib Akhtar likens himself to Brazilian icon Ronaldo Nazario if he swapped Pakistan cricket to play football</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2023,294 +2023,294 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Get the day-by-day Tarouba, Trinidad weather forecast and hourly rain probability for the West Indies vs Pakistan 1st Test at Brian Lara Cricket Academy.</t>
+          <t>Former Pakistan speedster Shoaib Akhtar claims he would have played like Brazilian legend Ronaldo Nazario had he chosen football over international cricket.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/tarouba-trinidad-weather-day-rain-chances-wi-vs-pak-1st-test-2026/c0c03fca2c4070682db8cb26</t>
+          <t>https://www.cricketnews.com/en/cricket/news/shoaib-akhtar-brazilian-ronaldo-nazario-pakistan-cricket-football/a8907afaa907e84e21f7aea7</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-07-25 12:26:43</t>
+          <t>2026-07-25 03:52:34</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>England to face Pakistan and Sri Lanka in tri-series</t>
+          <t>Tarouba, Trinidad weather forecast: Day-by-Day rain chances for West Indies vs Pakistan 1st Test 2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Matthew Henry - BBC Sport Journalist</t>
+          <t>Soham Mukherjee</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>England will play Pakistan and Sri Lanka in Lahore and Rawalpindi in a one-day international tri-series in October.</t>
+          <t>Get the day-by-day Tarouba, Trinidad weather forecast and hourly rain probability for the West Indies vs Pakistan 1st Test at Brian Lara Cricket Academy.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.bbc.com/sport/cricket/articles/c4g618j21xko?xtor=AL-72-%5Bpartner%5D-%5Byahoo.north.america%5D-%5Bheadline%5D-%5Bsport%5D-%5Bbizdev%5D-%5Bisapi%5D</t>
+          <t>https://www.cricketnews.com/en/cricket/news/tarouba-trinidad-weather-day-rain-chances-wi-vs-pak-1st-test-2026/c0c03fca2c4070682db8cb26</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-08-19 12:31:57</t>
+          <t>2026-07-25 12:26:43</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Jemimah Rodrigues hugs Pakistan captain Fatima Sana in The Hundred despite India’s strict 'no handshake' protocol</t>
+          <t>England to face Pakistan and Sri Lanka in tri-series</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Soham Mukherjee</t>
+          <t>Matthew Henry - BBC Sport Journalist</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Jemimah Rodrigues hugged Pakistan captain Fatima Sana after The Hundred match, setting aside Team India's official "no handshake" protocol. Watch the viral video.</t>
+          <t>England will play Pakistan and Sri Lanka in Lahore and Rawalpindi in a one-day international tri-series in October.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/jemimah-rodrigues-hugs-pakistan-fatima-sana-hundred-india-no-handshake/8b9d9a41a2f42d4d6b23eecc</t>
+          <t>https://www.bbc.com/sport/cricket/articles/c4g618j21xko?xtor=AL-72-%5Bpartner%5D-%5Byahoo.north.america%5D-%5Bheadline%5D-%5Bsport%5D-%5Bbizdev%5D-%5Bisapi%5D</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-07-31 04:00:23</t>
+          <t>2026-08-19 12:31:57</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Sri Lanka vs. Pakistan women prediction, lineups and betting tips for 1st T20I</t>
+          <t>Jemimah Rodrigues hugs Pakistan captain Fatima Sana in The Hundred despite India’s strict 'no handshake' protocol</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ajay Gandhar</t>
+          <t>Soham Mukherjee</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Sri Lanka Women host Pakistan Women in the first T20I of the tour. Get predictions, lineups and betting tips as Chamari Athapaththu looks to continue Sri Lanka's dominant run against a struggling Pakistan side.</t>
+          <t>Jemimah Rodrigues hugged Pakistan captain Fatima Sana after The Hundred match, setting aside Team India's official "no handshake" protocol. Watch the viral video.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.sportingnews.com/in/cricket/news/sri-lanka-vs-pakistan-women-prediction-lineups-betting-tips-1st-t20i/56459bba7ae133f3d72d79bb</t>
+          <t>https://www.cricketnews.com/en/cricket/news/jemimah-rodrigues-hugs-pakistan-fatima-sana-hundred-india-no-handshake/8b9d9a41a2f42d4d6b23eecc</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-07-30 14:10:01</t>
+          <t>2026-07-31 04:00:23</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Pakistan all-rounder handed two-year ban over visa misrepresentation: PCB says conduct tarnished PAK cricket's reputation</t>
+          <t>Sri Lanka vs. Pakistan women prediction, lineups and betting tips for 1st T20I</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Deepanjan Mitra</t>
+          <t>Ajay Gandhar</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Hamza Nazar's time with the Pakistan national team has been cut short before it even begins, after the bowler was banned for two years by the PCB for providing misleading visa information.</t>
+          <t>Sri Lanka Women host Pakistan Women in the first T20I of the tour. Get predictions, lineups and betting tips as Chamari Athapaththu looks to continue Sri Lanka's dominant run against a struggling Pakistan side.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/pakistan-all-rounder-two-year-ban-visa-pcb-reputation/2afdd7cfb7f450b7d245eb77</t>
+          <t>https://www.sportingnews.com/in/cricket/news/sri-lanka-vs-pakistan-women-prediction-lineups-betting-tips-1st-t20i/56459bba7ae133f3d72d79bb</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-08-07 08:32:21</t>
+          <t>2026-07-30 14:10:01</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Pakistan needs 18 runs against West Indies to win second test</t>
+          <t>Pakistan all-rounder handed two-year ban over visa misrepresentation: PCB says conduct tarnished PAK cricket's reputation</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Associated Press</t>
+          <t>Deepanjan Mitra</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Pakistan needs 18 more runs for a series-leveling victory against the West Indies in the second and final cricket test Wednesday as it seeks to end its eight-match losing streak away from home in test matches. First innings century-maker Abdullah Shafique was…</t>
+          <t>Hamza Nazar's time with the Pakistan national team has been cut short before it even begins, after the bowler was banned for two years by the PCB for providing misleading visa information.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/pakistan-needs-18-runs-against-162724450.html</t>
+          <t>https://www.cricketnews.com/en/cricket/news/pakistan-all-rounder-two-year-ban-visa-pcb-reputation/2afdd7cfb7f450b7d245eb77</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-08-05 16:27:24</t>
+          <t>2026-08-07 08:32:21</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>England vs. Pakistan prediction, lineups, pitch report for 1st test as Joe Root returns as captain</t>
+          <t>Pakistan needs 18 runs against West Indies to win second test</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Ajay Gandhar</t>
+          <t>Associated Press</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Joe Root returns as England captain for the Pakistan Test opener. Full prediction, team news and pitch report inside.</t>
+          <t>Pakistan needs 18 more runs for a series-leveling victory against the West Indies in the second and final cricket test Wednesday as it seeks to end its eight-match losing streak away from home in test matches. First innings century-maker Abdullah Shafique was…</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/play/england-vs-pakistan-prediction-lineups-pitch-report-1st-test-joe-root-returns-captain/327fc6a0c435faf04ca0f375</t>
+          <t>https://sports.yahoo.com/articles/pakistan-needs-18-runs-against-162724450.html</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-08-17 15:30:01</t>
+          <t>2026-08-05 16:27:24</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Only way India and Pakistan can meet at 2026 Asian Games cricket: Potential route to final, gold medal match in Aichi-Nagoya</t>
+          <t>England vs. Pakistan prediction, lineups, pitch report for 1st test as Joe Root returns as captain</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Deepanjan Mitra</t>
+          <t>Ajay Gandhar</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>With this year's Asian Games about to include cricket, fans across the subcontinent are excited to take a look at the India vs. Pakistan match in Japan, but there is only one way for them to meet.</t>
+          <t>Joe Root returns as England captain for the Pakistan Test opener. Full prediction, team news and pitch report inside.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/india-pakistan-meet-2026-asian-games-cricket-route-final-gold-medal/f100f9244c13dc31e2d904c1</t>
+          <t>https://www.cricketnews.com/en/cricket/play/england-vs-pakistan-prediction-lineups-pitch-report-1st-test-joe-root-returns-captain/327fc6a0c435faf04ca0f375</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-07-24 11:30:24</t>
+          <t>2026-08-17 15:30:01</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Greaves takes four wickets without a run as Pakistan trails West Indies by 44 runs in first test</t>
+          <t>Only way India and Pakistan can meet at 2026 Asian Games cricket: Potential route to final, gold medal match in Aichi-Nagoya</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Associated Press</t>
+          <t>Deepanjan Mitra</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Pakistan collapsed to 267-8 at lunch after Justin Greaves bowled four consecutive wicket maiden overs as West Indies made a strong comeback in the first cricket test on Monday. Greaves’ impeccable seam bowling led Pakistan to lose five wickets for 15 runs in …</t>
+          <t>With this year's Asian Games about to include cricket, fans across the subcontinent are excited to take a look at the India vs. Pakistan match in Japan, but there is only one way for them to meet.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://sports.yahoo.com/articles/greaves-takes-four-wickets-without-171636678.html</t>
+          <t>https://www.cricketnews.com/en/cricket/news/india-pakistan-meet-2026-asian-games-cricket-route-final-gold-medal/f100f9244c13dc31e2d904c1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-07-27 17:16:36</t>
+          <t>2026-07-24 11:30:24</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>''This is our culture': Fans react to 'typical' Pakistan collapse in 1st Test vs WI as Justin Greaves scalps 5-wicket haul</t>
+          <t>Greaves takes four wickets without a run as Pakistan trails West Indies by 44 runs in first test</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Deepanjan Mitra</t>
+          <t>Associated Press</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Pakistan faces one of their typical batting collapses as a five-wicket haul by Justin Greaves while fans do not give the team any respite with their blunt takes.</t>
+          <t>Pakistan collapsed to 267-8 at lunch after Justin Greaves bowled four consecutive wicket maiden overs as West Indies made a strong comeback in the first cricket test on Monday. Greaves’ impeccable seam bowling led Pakistan to lose five wickets for 15 runs in …</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/fans-react-pakistan-collapse-1st-test-vs-wi-justin-greaves-5-wicket-haul/48d5205a9da1ebf81560915e</t>
+          <t>https://sports.yahoo.com/articles/greaves-takes-four-wickets-without-171636678.html</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-07-27 18:26:32</t>
+          <t>2026-07-27 17:16:36</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Babar Azam Test centuries: Full career stats detailed as Pakistan captain on the verge of scoring first Test 100 in four years</t>
+          <t>''This is our culture': Fans react to 'typical' Pakistan collapse in 1st Test vs WI as Justin Greaves scalps 5-wicket haul</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Soham Mukherjee</t>
+          <t>Deepanjan Mitra</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Explore Babar Azam's full Test career stats and list of centuries as the Pakistan captain closes in on his first Test 100 since 2022 vs West Indies.</t>
+          <t>Pakistan faces one of their typical batting collapses as a five-wicket haul by Justin Greaves while fans do not give the team any respite with their blunt takes.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/babar-azam-test-centuries-full-career-stats/5cfa0950af88fc6f8dad4787</t>
+          <t>https://www.cricketnews.com/en/cricket/news/fans-react-pakistan-collapse-1st-test-vs-wi-justin-greaves-5-wicket-haul/48d5205a9da1ebf81560915e</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-08-04 03:55:46</t>
+          <t>2026-07-27 18:26:32</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>'We pull him down': Azhar Mahmood slams treatment of Babar Azam &amp; cites 'lack of respect' for the Pakistan captain</t>
+          <t>Babar Azam Test centuries: Full career stats detailed as Pakistan captain on the verge of scoring first Test 100 in four years</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2320,51 +2320,51 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Azhar Mahmood defended Babar Azam, revealing how harsh criticism from former players affected him and why Pakistan must respect its only superstar.</t>
+          <t>Explore Babar Azam's full Test career stats and list of centuries as the Pakistan captain closes in on his first Test 100 since 2022 vs West Indies.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/azhar-mahmood-babar-azam-lack-respect-pakistan-captain/132e4501d5516aaa7b4aac2e</t>
+          <t>https://www.cricketnews.com/en/cricket/news/babar-azam-test-centuries-full-career-stats/5cfa0950af88fc6f8dad4787</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-08-17 16:50:43</t>
+          <t>2026-08-04 03:55:46</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Where to watch Sri Lanka vs Pakistan live stream, TV channel, start time and lineups for 1st women's ODI</t>
+          <t>'We pull him down': Azhar Mahmood slams treatment of Babar Azam &amp; cites 'lack of respect' for the Pakistan captain</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Anselm Noronha</t>
+          <t>Soham Mukherjee</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>All the details for Sri Lanka Women vs Pakistan Women 1st ODI, including broadcast info, start time and squads.</t>
+          <t>Azhar Mahmood defended Babar Azam, revealing how harsh criticism from former players affected him and why Pakistan must respect its only superstar.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.sportingnews.com/in/cricket/news/watch-sri-lanka-pakistan-live-stream-tv-channel-start-time-lineups-1st-womens-odi/3da9ce8437c518dcd27d8392</t>
+          <t>https://www.cricketnews.com/en/cricket/news/azhar-mahmood-babar-azam-lack-respect-pakistan-captain/132e4501d5516aaa7b4aac2e</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-07-22 17:30:01</t>
+          <t>2026-08-17 16:50:43</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Lancashire bring in Pakistan spinner Noman</t>
+          <t>Send your cricket data questions to BBC Sport &amp; CricViz</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2374,24 +2374,24 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Lancashire sign Pakistan spinner Noman Ali for the final six games of the County Championship season.</t>
+          <t>Send your cricket data questions to BBC Sport and we will get CricViz to answer a selection of them.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.bbc.com/sport/cricket/articles/c9d893pzv34o?xtor=AL-72-%5Bpartner%5D-%5Byahoo.north.america%5D-%5Bheadline%5D-%5Bsport%5D-%5Bbizdev%5D-%5Bisapi%5D</t>
+          <t>https://www.bbc.com/sport/cricket/articles/cz6459x3zw0o?xtor=AL-72-%5Bpartner%5D-%5Byahoo.north.america%5D-%5Bheadline%5D-%5Bsport%5D-%5Bbizdev%5D-%5Bisapi%5D</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-08-06 10:36:10</t>
+          <t>2026-08-19 16:05:41</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>WI vs PAK 1st Test session timings: Start times, lunch and tea breaks for West Indies vs Pakistan 2026 at Tarouba</t>
+          <t>Where to watch Sri Lanka vs Pakistan live stream, TV channel, start time and lineups for 1st women's ODI</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2401,105 +2401,105 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Pakistan begin their 2026 Test series against West Indies at Tarouba. Here's the full daily schedule, including match start times and the lunch and tea intervals for the opening Test.</t>
+          <t>All the details for Sri Lanka Women vs Pakistan Women 1st ODI, including broadcast info, start time and squads.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/wi-vs-pak-1st-test-session-timings-start-times-lunch-tea-break/fd75e38d0fa41faaeba76748</t>
+          <t>https://www.sportingnews.com/in/cricket/news/watch-sri-lanka-pakistan-live-stream-tv-channel-start-time-lineups-1st-womens-odi/3da9ce8437c518dcd27d8392</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-07-25 12:25:14</t>
+          <t>2026-07-22 17:30:01</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Explained: Why Michael Vaughan is unhappy that Stephen Fleming will join England team after Pakistan Test series</t>
+          <t>Lancashire bring in Pakistan spinner Noman</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Soham Mukherjee</t>
+          <t>BBC</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Former England captain Michael Vaughan has criticised Stephen Fleming's decision to join the Test setup only after the upcoming Pakistan series. Read why.</t>
+          <t>Lancashire sign Pakistan spinner Noman Ali for the final six games of the County Championship season.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/why-michael-vaughan-unhappy-stephen-fleming-england-pakistan-test-series/22aee1e3b1b7ce4f8764dcf0</t>
+          <t>https://www.bbc.com/sport/cricket/articles/c9d893pzv34o?xtor=AL-72-%5Bpartner%5D-%5Byahoo.north.america%5D-%5Bheadline%5D-%5Bsport%5D-%5Bbizdev%5D-%5Bisapi%5D</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-07-30 16:21:51</t>
+          <t>2026-08-06 10:36:10</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>How to watch ENG vs PAK Test series 2026 live: Start time, TV channels and streaming details</t>
+          <t>WI vs PAK 1st Test session timings: Start times, lunch and tea breaks for West Indies vs Pakistan 2026 at Tarouba</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Deepanjan Mitra</t>
+          <t>Anselm Noronha</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>With the first Test between England and Pakistan just two days away, here's how you can watch the game live without missing a single ball.</t>
+          <t>Pakistan begin their 2026 Test series against West Indies at Tarouba. Here's the full daily schedule, including match start times and the lunch and tea intervals for the opening Test.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/watch-eng-vs-pak-test-series-2026-live-start-time-tv-channels-streaming/a974c768210e34aa168476ad</t>
+          <t>https://www.cricketnews.com/en/cricket/news/wi-vs-pak-1st-test-session-timings-start-times-lunch-tea-break/fd75e38d0fa41faaeba76748</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-08-18 09:52:21</t>
+          <t>2026-07-25 12:25:14</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Pakistan to tour England for five-match ODI series ahead of 2027 Cricket World Cup</t>
+          <t>Explained: Why Michael Vaughan is unhappy that Stephen Fleming will join England team after Pakistan Test series</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Unknown Author</t>
+          <t>Soham Mukherjee</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Pakistan will tour England for a five-match ODI series in May 2027. This series will serve as crucial preparation for the ICC Men's Cricket World Cup 2027. The World Cup is scheduled to be held later that year in October and November. The tour begins in South…</t>
+          <t>Former England captain Michael Vaughan has criticised Stephen Fleming's decision to join the Test setup only after the upcoming Pakistan series. Read why.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://consent.yahoo.com/v2/collectConsent?sessionId=1_cc-session_f0e186ea-cfc9-4800-96fa-dd23d961f25f</t>
+          <t>https://www.cricketnews.com/en/cricket/news/why-michael-vaughan-unhappy-stephen-fleming-england-pakistan-test-series/22aee1e3b1b7ce4f8764dcf0</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026-07-23 15:28:00</t>
+          <t>2026-07-30 16:21:51</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Babar Azam injury: Availability and latest update on Pakistan captain ahead of 1st Test vs England at Leeds</t>
+          <t>How to watch ENG vs PAK Test series 2026 live: Start time, TV channels and streaming details</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2509,78 +2509,78 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>With injury rumours swirling around Pakistani skipper Babar Azam for the first Test against England, latest updates believe that he would play the match.</t>
+          <t>With the first Test between England and Pakistan just two days away, here's how you can watch the game live without missing a single ball.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/babar-azam-injury-availability-latest-update-pakistan-england/6ed9ebc3291d57a5e18001ca</t>
+          <t>https://www.cricketnews.com/en/cricket/news/watch-eng-vs-pak-test-series-2026-live-start-time-tv-channels-streaming/a974c768210e34aa168476ad</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-08-15 16:44:10</t>
+          <t>2026-08-18 09:52:21</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Babar Azam's last Test century: Pakistan star's hundred drought in Test cricket explained</t>
+          <t>Pakistan to tour England for five-match ODI series ahead of 2027 Cricket World Cup</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Deepanjan Mitra</t>
+          <t>Unknown Author</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>After getting run out for 88 against the West Indies in the second Test, Babar Azam has now gone 17 Test matches without scoring a century.</t>
+          <t>Pakistan will tour England for a five-match ODI series in May 2027. This series will serve as crucial preparation for the ICC Men's Cricket World Cup 2027. The World Cup is scheduled to be held later that year in October and November. The tour begins in South…</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/babar-azam-last-test-century-pakistan-hundred-drought-test-cricket/205a9ea7e3414fe6b605c1b6</t>
+          <t>https://consent.yahoo.com/v2/collectConsent?sessionId=1_cc-session_f0e186ea-cfc9-4800-96fa-dd23d961f25f</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-08-04 18:49:57</t>
+          <t>2026-07-23 15:28:00</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>'Not your job': Usman Tariq's bold message to opponents over questions being raised on controversial bowling action</t>
+          <t>Babar Azam injury: Availability and latest update on Pakistan captain ahead of 1st Test vs England at Leeds</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Anselm Noronha</t>
+          <t>Deepanjan Mitra</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Pakistan spinner Usman Tariq has hit back at opponents questioning his bowling action, insisting that only umpires and officials have the authority to judge its legality.</t>
+          <t>With injury rumours swirling around Pakistani skipper Babar Azam for the first Test against England, latest updates believe that he would play the match.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/usman-tariq-message-opponents-questions-raised-controversial-action/2b629b67a9020f2e0efe8771</t>
+          <t>https://www.cricketnews.com/en/cricket/news/babar-azam-injury-availability-latest-update-pakistan-england/6ed9ebc3291d57a5e18001ca</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-07-27 09:03:31</t>
+          <t>2026-08-15 16:44:10</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ENG vs PAK 1st Test session timings: Start times, lunch and tea breaks for Pakistan tour of England at Headingley</t>
+          <t>Babar Azam's last Test century: Pakistan star's hundred drought in Test cricket explained</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2590,51 +2590,51 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>With the England vs. Pakistan 1st test match underway, here's all the session timings along with the lunch and tea breaks</t>
+          <t>After getting run out for 88 against the West Indies in the second Test, Babar Azam has now gone 17 Test matches without scoring a century.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/eng-vs-pak-1st-test-session-timings-start-times-lunch-tea-breaks/cb6ad23faa3301bc96d2b6c8</t>
+          <t>https://www.cricketnews.com/en/cricket/news/babar-azam-last-test-century-pakistan-hundred-drought-test-cricket/205a9ea7e3414fe6b605c1b6</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2026-08-19 02:46:56</t>
+          <t>2026-08-04 18:49:57</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>West Indies triumph as Pakistan suffer 8th consecutive overseas Test defeat! When did Babar Azam last win a Test abroad?</t>
+          <t>'Not your job': Usman Tariq's bold message to opponents over questions being raised on controversial bowling action</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Soham Mukherjee</t>
+          <t>Anselm Noronha</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Pakistan suffered their eighth consecutive away Test defeat in Trinidad against the West Indies. Discover how their historic overseas losing streak unfolded.</t>
+          <t>Pakistan spinner Usman Tariq has hit back at opponents questioning his bowling action, insisting that only umpires and officials have the authority to judge its legality.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/west-indies-pakistan-overseas-test-defeat-babar-azam-last-win/8703256c9ee3d0bd1a5546e4</t>
+          <t>https://www.cricketnews.com/en/cricket/news/usman-tariq-message-opponents-questions-raised-controversial-action/2b629b67a9020f2e0efe8771</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-07-29 04:41:44</t>
+          <t>2026-07-27 09:03:31</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>England's new Test captain and head coach for Pakistan series: Likely candidates to take over after Ben Stokes and Brendon McCullum</t>
+          <t>ENG vs PAK 1st Test session timings: Start times, lunch and tea breaks for Pakistan tour of England at Headingley</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2644,44 +2644,44 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>With Ben Stokes and Brendon McCullum both out of the England dressing room, here's a look at the likely candidates ahead of the upcoming series against Pakistan.</t>
+          <t>With the England vs. Pakistan 1st test match underway, here's all the session timings along with the lunch and tea breaks</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://www.cricketnews.com/en/cricket/news/englands-test-captain-head-coach-pakistan-series/2106ec337adc465fab4f3af5</t>
+          <t>https://www.cricketnews.com/en/cricket/news/eng-vs-pak-1st-test-session-timings-start-times-lunch-tea-breaks/cb6ad23faa3301bc96d2b6c8</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-07-24 14:36:41</t>
+          <t>2026-08-19 02:46:56</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Cricket at Asian Games 2026: India women take on Japan in quarterfinals</t>
+          <t>England's new Test captain and head coach for Pakistan series: Likely candidates to take over after Ben Stokes and Brendon McCullum</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Soham Mukherjee</t>
+          <t>Deepanjan Mitra</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>India Women take on Japan in the quarterfinals of cricket at the 2026 Asian Games. Get the match schedule, key players, and knockout scenario.</t>
+          <t>With Ben Stokes and Brendon McCullum both out of the England dressing room, here's a look at the likely candidates ahead of the upcoming series against Pakistan.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://www.sportingnews.com/in/cricket/news/cricket-asian-games-2026-india-women-japan-quarterfinals/7ea826865a7f8237ebb75d8c</t>
+          <t>https://www.cricketnews.com/en/cricket/news/englands-test-captain-head-coach-pakistan-series/2106ec337adc465fab4f3af5</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-07-24 07:35:45</t>
+          <t>2026-07-24 14:36:41</t>
         </is>
       </c>
     </row>

</xml_diff>